<commit_message>
Phase 9: Data injection pipeline - UI to DB v3: apart from api everyhting almost ready
</commit_message>
<xml_diff>
--- a/Backend/extra_datasource/Data_Ingestion/PPS Products Cycle Time 05-02-2026.xlsx
+++ b/Backend/extra_datasource/Data_Ingestion/PPS Products Cycle Time 05-02-2026.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Item code review" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$161</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
@@ -421,7 +421,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="282">
   <si>
     <t>Sl No</t>
   </si>
@@ -549,9 +549,6 @@
     <t>PUREPRINT WF</t>
   </si>
   <si>
-    <t>MTPPBULK00000013</t>
-  </si>
-  <si>
     <t>PUREPRINT WHITE NC PLUS</t>
   </si>
   <si>
@@ -615,9 +612,6 @@
     <t>PURONAL WET NF 60 CONC-E</t>
   </si>
   <si>
-    <t>TDBNAX000PUSY010</t>
-  </si>
-  <si>
     <t>PURETHANE AM 501</t>
   </si>
   <si>
@@ -627,9 +621,6 @@
     <t>PURETHANE IA 403</t>
   </si>
   <si>
-    <t>TDBNAX000PUSY017</t>
-  </si>
-  <si>
     <t>PURETHANE IA 403 UP</t>
   </si>
   <si>
@@ -645,9 +636,6 @@
     <t>PUREISO MP 20</t>
   </si>
   <si>
-    <t>MGCNAX000PMDI021</t>
-  </si>
-  <si>
     <t>PUREISO TM 20</t>
   </si>
   <si>
@@ -831,9 +819,6 @@
     <t>Not availability of  QC person is not considered</t>
   </si>
   <si>
-    <t>TDBNAX000PUSY016</t>
-  </si>
-  <si>
     <t>PURETHANE IA 403 SPL</t>
   </si>
   <si>
@@ -1267,6 +1252,21 @@
   </si>
   <si>
     <t>Proposed code for PURETHANE 5290/1. No product 52090/1 exists in CRM; PSM makes 5290/1. Plant to confirm the name is a typo.</t>
+  </si>
+  <si>
+    <t>MTPPHDCB00050197</t>
+  </si>
+  <si>
+    <t>MGCMSN210PUSY008</t>
+  </si>
+  <si>
+    <t>MGCMSN210PUSY004</t>
+  </si>
+  <si>
+    <t>MGCMSN230PMDI020</t>
+  </si>
+  <si>
+    <t>MGCMSN210PUSY005</t>
   </si>
 </sst>
 </file>
@@ -1706,7 +1706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W162"/>
+  <dimension ref="A1:W161"/>
   <sheetFormatPr defaultRowHeight="13" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" style="19" bestFit="1" customWidth="1"/>
@@ -2358,10 +2358,10 @@
         <v>22</v>
       </c>
       <c r="C10" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>43</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>25</v>
@@ -2426,13 +2426,13 @@
         <v>22</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="F11" s="3">
         <v>200</v>
@@ -2494,13 +2494,13 @@
         <v>22</v>
       </c>
       <c r="C12" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>48</v>
-      </c>
       <c r="E12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F12" s="3">
         <v>200</v>
@@ -2562,13 +2562,13 @@
         <v>22</v>
       </c>
       <c r="C13" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="18" t="s">
-        <v>50</v>
-      </c>
       <c r="E13" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F13" s="3">
         <v>200</v>
@@ -2630,13 +2630,13 @@
         <v>22</v>
       </c>
       <c r="C14" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="F14" s="3">
         <v>1000</v>
@@ -2698,13 +2698,13 @@
         <v>22</v>
       </c>
       <c r="C15" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="E15" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="3">
         <v>1000</v>
@@ -2766,13 +2766,13 @@
         <v>22</v>
       </c>
       <c r="C16" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="E16" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F16" s="3">
         <v>1000</v>
@@ -2834,13 +2834,13 @@
         <v>22</v>
       </c>
       <c r="C17" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="E17" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F17" s="3">
         <v>1000</v>
@@ -2902,13 +2902,13 @@
         <v>22</v>
       </c>
       <c r="C18" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="E18" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F18" s="3">
         <v>1000</v>
@@ -2970,13 +2970,13 @@
         <v>22</v>
       </c>
       <c r="C19" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="E19" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" s="3">
         <v>1000</v>
@@ -3038,13 +3038,13 @@
         <v>22</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>64</v>
+        <v>278</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F20" s="3">
         <v>1000</v>
@@ -3107,13 +3107,13 @@
         <v>22</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F21" s="3">
         <v>1000</v>
@@ -3176,13 +3176,13 @@
         <v>22</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>68</v>
+        <v>279</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F22" s="3">
         <v>1000</v>
@@ -3245,13 +3245,13 @@
         <v>22</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F23" s="3">
         <v>1000</v>
@@ -3314,13 +3314,13 @@
         <v>22</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F24" s="3">
         <v>1000</v>
@@ -3383,13 +3383,13 @@
         <v>22</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>74</v>
+        <v>280</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F25" s="3">
         <v>1000</v>
@@ -3452,13 +3452,13 @@
         <v>22</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F26" s="3">
         <v>1000</v>
@@ -3521,13 +3521,13 @@
         <v>22</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F27" s="3">
         <v>1000</v>
@@ -3590,13 +3590,13 @@
         <v>22</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F28" s="3">
         <v>1000</v>
@@ -3659,13 +3659,13 @@
         <v>22</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F29" s="3">
         <v>1000</v>
@@ -3728,13 +3728,13 @@
         <v>22</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F30" s="3">
         <v>1000</v>
@@ -3797,13 +3797,13 @@
         <v>22</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F31" s="3">
         <v>1000</v>
@@ -3866,13 +3866,13 @@
         <v>22</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F32" s="3">
         <v>1000</v>
@@ -3935,13 +3935,13 @@
         <v>22</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F33" s="3">
         <v>1000</v>
@@ -4004,13 +4004,13 @@
         <v>22</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F34" s="3">
         <v>1000</v>
@@ -4073,13 +4073,13 @@
         <v>22</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F35" s="3">
         <v>1000</v>
@@ -4142,13 +4142,13 @@
         <v>22</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F36" s="3">
         <v>1000</v>
@@ -4211,13 +4211,13 @@
         <v>22</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F37" s="3">
         <v>1000</v>
@@ -4280,13 +4280,13 @@
         <v>22</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F38" s="3">
         <v>1000</v>
@@ -4349,13 +4349,13 @@
         <v>22</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F39" s="3">
         <v>1000</v>
@@ -4418,13 +4418,13 @@
         <v>22</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F40" s="3">
         <v>1000</v>
@@ -4487,13 +4487,13 @@
         <v>22</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F41" s="3">
         <v>1000</v>
@@ -4556,13 +4556,13 @@
         <v>22</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F42" s="3">
         <v>1000</v>
@@ -4625,13 +4625,13 @@
         <v>22</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F43" s="3">
         <v>1000</v>
@@ -4694,13 +4694,13 @@
         <v>22</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F44" s="3">
         <v>1000</v>
@@ -4763,13 +4763,13 @@
         <v>22</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F45" s="6">
         <v>1000</v>
@@ -4832,13 +4832,13 @@
         <v>22</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F46" s="6">
         <v>1000</v>
@@ -4901,13 +4901,13 @@
         <v>22</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F47" s="6">
         <v>1000</v>
@@ -4922,7 +4922,7 @@
         <v>1</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K47" s="3">
         <v>2</v>
@@ -4970,13 +4970,13 @@
         <v>22</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F48" s="6">
         <v>1000</v>
@@ -5039,13 +5039,13 @@
         <v>22</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>64</v>
+        <v>278</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F49" s="3">
         <v>10000</v>
@@ -5060,7 +5060,7 @@
         <v>210</v>
       </c>
       <c r="J49" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K49" s="3">
         <v>8</v>
@@ -5105,13 +5105,13 @@
         <v>22</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F50" s="3">
         <v>10000</v>
@@ -5126,7 +5126,7 @@
         <v>210</v>
       </c>
       <c r="J50" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K50" s="3">
         <v>8</v>
@@ -5171,13 +5171,13 @@
         <v>22</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F51" s="3">
         <v>10000</v>
@@ -5192,7 +5192,7 @@
         <v>210</v>
       </c>
       <c r="J51" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K51" s="3">
         <v>8</v>
@@ -5237,13 +5237,13 @@
         <v>22</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F52" s="3">
         <v>10000</v>
@@ -5258,7 +5258,7 @@
         <v>210</v>
       </c>
       <c r="J52" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K52" s="3">
         <v>8</v>
@@ -5303,13 +5303,13 @@
         <v>22</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D53" s="18" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F53" s="3">
         <v>10000</v>
@@ -5324,7 +5324,7 @@
         <v>210</v>
       </c>
       <c r="J53" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K53" s="3">
         <v>8</v>
@@ -5369,13 +5369,13 @@
         <v>22</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D54" s="18" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F54" s="3">
         <v>10000</v>
@@ -5390,7 +5390,7 @@
         <v>210</v>
       </c>
       <c r="J54" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K54" s="3">
         <v>8</v>
@@ -5435,13 +5435,13 @@
         <v>22</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D55" s="18" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F55" s="3">
         <v>10000</v>
@@ -5456,7 +5456,7 @@
         <v>210</v>
       </c>
       <c r="J55" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K55" s="3">
         <v>8</v>
@@ -5501,13 +5501,13 @@
         <v>22</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F56" s="3">
         <v>7500</v>
@@ -5522,7 +5522,7 @@
         <v>210</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K56" s="3">
         <v>8</v>
@@ -5557,7 +5557,7 @@
         <v>51</v>
       </c>
       <c r="U56" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V56" s="18"/>
     </row>
@@ -5569,13 +5569,13 @@
         <v>22</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>136</v>
+        <v>281</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F57" s="3">
         <v>7500</v>
@@ -5590,7 +5590,7 @@
         <v>210</v>
       </c>
       <c r="J57" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K57" s="3">
         <v>8</v>
@@ -5625,7 +5625,7 @@
         <v>51</v>
       </c>
       <c r="U57" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V57" s="18"/>
     </row>
@@ -5637,13 +5637,13 @@
         <v>22</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>68</v>
+        <v>279</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F58" s="3">
         <v>7500</v>
@@ -5658,7 +5658,7 @@
         <v>210</v>
       </c>
       <c r="J58" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K58" s="3">
         <v>8</v>
@@ -5693,7 +5693,7 @@
         <v>51</v>
       </c>
       <c r="U58" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V58" s="18"/>
     </row>
@@ -5705,13 +5705,13 @@
         <v>22</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F59" s="3">
         <v>5000</v>
@@ -5761,7 +5761,7 @@
         <v>35.702380952380949</v>
       </c>
       <c r="U59" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="V59" s="18"/>
     </row>
@@ -5773,13 +5773,13 @@
         <v>22</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F60" s="3">
         <v>5000</v>
@@ -5829,7 +5829,7 @@
         <v>35.702380952380949</v>
       </c>
       <c r="U60" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="V60" s="18"/>
     </row>
@@ -5841,13 +5841,13 @@
         <v>22</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F61" s="3">
         <v>5000</v>
@@ -5897,7 +5897,7 @@
         <v>35.702380952380949</v>
       </c>
       <c r="U61" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="V61" s="18"/>
     </row>
@@ -5909,13 +5909,13 @@
         <v>22</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F62" s="3">
         <v>5000</v>
@@ -5965,7 +5965,7 @@
         <v>36.202380952380949</v>
       </c>
       <c r="U62" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="V62" s="18"/>
     </row>
@@ -5977,13 +5977,13 @@
         <v>22</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D63" s="18" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F63" s="3">
         <v>5000</v>
@@ -6033,7 +6033,7 @@
         <v>36.202380952380949</v>
       </c>
       <c r="U63" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="V63" s="18"/>
     </row>
@@ -6045,13 +6045,13 @@
         <v>22</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F64" s="3">
         <v>5000</v>
@@ -6111,13 +6111,13 @@
         <v>22</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F65" s="3">
         <v>5000</v>
@@ -6177,13 +6177,13 @@
         <v>22</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F66" s="3">
         <v>2000</v>
@@ -6233,7 +6233,7 @@
         <v>15.8</v>
       </c>
       <c r="U66" s="18" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="V66" s="18"/>
     </row>
@@ -6245,13 +6245,13 @@
         <v>22</v>
       </c>
       <c r="C67" s="20" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F67" s="3">
         <v>1000</v>
@@ -6266,7 +6266,7 @@
         <v>70</v>
       </c>
       <c r="J67" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K67" s="3">
         <v>3</v>
@@ -6311,13 +6311,13 @@
         <v>22</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D68" s="18" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F68" s="3">
         <v>1000</v>
@@ -6332,7 +6332,7 @@
         <v>50</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K68" s="3">
         <v>3</v>
@@ -6377,13 +6377,13 @@
         <v>22</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F69" s="3">
         <v>1000</v>
@@ -6398,7 +6398,7 @@
         <v>70</v>
       </c>
       <c r="J69" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K69" s="3">
         <v>3</v>
@@ -6443,13 +6443,13 @@
         <v>22</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F70" s="3">
         <v>1000</v>
@@ -6464,7 +6464,7 @@
         <v>1000</v>
       </c>
       <c r="J70" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K70" s="3">
         <v>3</v>
@@ -6509,13 +6509,13 @@
         <v>22</v>
       </c>
       <c r="C71" s="20" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F71" s="3">
         <v>1000</v>
@@ -6530,7 +6530,7 @@
         <v>70</v>
       </c>
       <c r="J71" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K71" s="3">
         <v>3</v>
@@ -6575,13 +6575,13 @@
         <v>22</v>
       </c>
       <c r="C72" s="20" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F72" s="3">
         <v>1000</v>
@@ -6596,7 +6596,7 @@
         <v>120</v>
       </c>
       <c r="J72" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K72" s="3">
         <v>3</v>
@@ -6641,13 +6641,13 @@
         <v>22</v>
       </c>
       <c r="C73" s="20" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F73" s="3">
         <v>1000</v>
@@ -6662,7 +6662,7 @@
         <v>50</v>
       </c>
       <c r="J73" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K73" s="3">
         <v>3</v>
@@ -6707,13 +6707,13 @@
         <v>22</v>
       </c>
       <c r="C74" s="20" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D74" s="18" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F74" s="3">
         <v>6000</v>
@@ -6773,13 +6773,13 @@
         <v>22</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F75" s="3">
         <v>6000</v>
@@ -6839,13 +6839,13 @@
         <v>22</v>
       </c>
       <c r="C76" s="20" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D76" s="18" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F76" s="3">
         <v>6000</v>
@@ -6905,13 +6905,13 @@
         <v>22</v>
       </c>
       <c r="C77" s="20" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D77" s="18" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F77" s="3">
         <v>6000</v>
@@ -6971,13 +6971,13 @@
         <v>22</v>
       </c>
       <c r="C78" s="20" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D78" s="18" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F78" s="3">
         <v>6000</v>
@@ -7037,13 +7037,13 @@
         <v>22</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F79" s="3">
         <v>6000</v>
@@ -7103,13 +7103,13 @@
         <v>22</v>
       </c>
       <c r="C80" s="20" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D80" s="18" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F80" s="3">
         <v>6000</v>
@@ -7169,13 +7169,13 @@
         <v>22</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F81" s="3">
         <v>6000</v>
@@ -7235,13 +7235,13 @@
         <v>22</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D82" s="18" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F82" s="3">
         <v>6000</v>
@@ -7301,13 +7301,13 @@
         <v>22</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F83" s="3">
         <v>6000</v>
@@ -7367,13 +7367,13 @@
         <v>22</v>
       </c>
       <c r="C84" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D84" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D84" s="18" t="s">
-        <v>52</v>
-      </c>
       <c r="E84" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F84" s="3">
         <v>6000</v>
@@ -7433,13 +7433,13 @@
         <v>22</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F85" s="3">
         <v>6000</v>
@@ -7499,13 +7499,13 @@
         <v>22</v>
       </c>
       <c r="C86" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="D86" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D86" s="18" t="s">
-        <v>55</v>
-      </c>
       <c r="E86" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F86" s="3">
         <v>6000</v>
@@ -7565,13 +7565,13 @@
         <v>22</v>
       </c>
       <c r="C87" s="20" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F87" s="3">
         <v>6000</v>
@@ -7631,13 +7631,13 @@
         <v>22</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="D88" s="18" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F88" s="3">
         <v>6000</v>
@@ -7697,13 +7697,13 @@
         <v>22</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F89" s="3">
         <v>6000</v>
@@ -7763,13 +7763,13 @@
         <v>22</v>
       </c>
       <c r="C90" s="20" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="D90" s="18" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F90" s="3">
         <v>6000</v>
@@ -7829,13 +7829,13 @@
         <v>22</v>
       </c>
       <c r="C91" s="20" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F91" s="3">
         <v>6000</v>
@@ -7895,13 +7895,13 @@
         <v>22</v>
       </c>
       <c r="C92" s="20" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D92" s="18" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F92" s="3">
         <v>6000</v>
@@ -7961,13 +7961,13 @@
         <v>22</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D93" s="18" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F93" s="3">
         <v>6000</v>
@@ -8027,13 +8027,13 @@
         <v>22</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D94" s="18" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F94" s="3">
         <v>6000</v>
@@ -8093,13 +8093,13 @@
         <v>22</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F95" s="3">
         <v>6000</v>
@@ -8159,13 +8159,13 @@
         <v>22</v>
       </c>
       <c r="C96" s="20" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D96" s="18" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F96" s="3">
         <v>6000</v>
@@ -8225,13 +8225,13 @@
         <v>22</v>
       </c>
       <c r="C97" s="20" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D97" s="18" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F97" s="3">
         <v>6000</v>
@@ -8291,13 +8291,13 @@
         <v>22</v>
       </c>
       <c r="C98" s="20" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D98" s="18" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F98" s="3">
         <v>6000</v>
@@ -8357,13 +8357,13 @@
         <v>22</v>
       </c>
       <c r="C99" s="20" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D99" s="18" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F99" s="3">
         <v>6000</v>
@@ -8423,13 +8423,13 @@
         <v>22</v>
       </c>
       <c r="C100" s="20" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D100" s="18" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F100" s="3">
         <v>6000</v>
@@ -8489,13 +8489,13 @@
         <v>22</v>
       </c>
       <c r="C101" s="20" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D101" s="18" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F101" s="3">
         <v>6000</v>
@@ -8555,13 +8555,13 @@
         <v>22</v>
       </c>
       <c r="C102" s="20" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D102" s="18" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F102" s="3">
         <v>6000</v>
@@ -8621,13 +8621,13 @@
         <v>22</v>
       </c>
       <c r="C103" s="20" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F103" s="3">
         <v>6000</v>
@@ -8687,13 +8687,13 @@
         <v>22</v>
       </c>
       <c r="C104" s="20" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F104" s="3">
         <v>6000</v>
@@ -8708,7 +8708,7 @@
         <v>50</v>
       </c>
       <c r="J104" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K104" s="3">
         <v>3</v>
@@ -8743,7 +8743,7 @@
         <v>21</v>
       </c>
       <c r="U104" s="4" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="V104" s="4"/>
     </row>
@@ -8755,13 +8755,13 @@
         <v>22</v>
       </c>
       <c r="C105" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D105" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D105" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="E105" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F105" s="3">
         <v>6000</v>
@@ -8776,7 +8776,7 @@
         <v>50</v>
       </c>
       <c r="J105" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K105" s="3">
         <v>3</v>
@@ -8811,7 +8811,7 @@
         <v>21</v>
       </c>
       <c r="U105" s="4" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="V105" s="4"/>
     </row>
@@ -8823,13 +8823,13 @@
         <v>22</v>
       </c>
       <c r="C106" s="20" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F106" s="3">
         <v>6000</v>
@@ -8844,7 +8844,7 @@
         <v>50</v>
       </c>
       <c r="J106" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K106" s="3">
         <v>2</v>
@@ -8889,13 +8889,13 @@
         <v>22</v>
       </c>
       <c r="C107" s="20" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F107" s="3">
         <v>6000</v>
@@ -8910,7 +8910,7 @@
         <v>1000</v>
       </c>
       <c r="J107" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K107" s="3">
         <v>2</v>
@@ -8955,13 +8955,13 @@
         <v>22</v>
       </c>
       <c r="C108" s="20" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F108" s="3">
         <v>6000</v>
@@ -8976,7 +8976,7 @@
         <v>50</v>
       </c>
       <c r="J108" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K108" s="3">
         <v>2</v>
@@ -9011,7 +9011,7 @@
         <v>19</v>
       </c>
       <c r="U108" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V108" s="4"/>
     </row>
@@ -9023,13 +9023,13 @@
         <v>22</v>
       </c>
       <c r="C109" s="20" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F109" s="3">
         <v>6000</v>
@@ -9044,7 +9044,7 @@
         <v>1000</v>
       </c>
       <c r="J109" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K109" s="3">
         <v>2</v>
@@ -9089,13 +9089,13 @@
         <v>22</v>
       </c>
       <c r="C110" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D110" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D110" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="E110" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F110" s="3">
         <v>6000</v>
@@ -9110,7 +9110,7 @@
         <v>50</v>
       </c>
       <c r="J110" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K110" s="3">
         <v>2</v>
@@ -9145,7 +9145,7 @@
         <v>19</v>
       </c>
       <c r="U110" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V110" s="4"/>
     </row>
@@ -9157,13 +9157,13 @@
         <v>22</v>
       </c>
       <c r="C111" s="20" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D111" s="13" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F111" s="3">
         <v>6000</v>
@@ -9178,7 +9178,7 @@
         <v>50</v>
       </c>
       <c r="J111" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K111" s="3">
         <v>2</v>
@@ -9213,7 +9213,7 @@
         <v>17</v>
       </c>
       <c r="U111" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V111" s="4"/>
     </row>
@@ -9225,13 +9225,13 @@
         <v>22</v>
       </c>
       <c r="C112" s="20" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F112" s="3">
         <v>6000</v>
@@ -9246,7 +9246,7 @@
         <v>50</v>
       </c>
       <c r="J112" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K112" s="3">
         <v>2</v>
@@ -9281,7 +9281,7 @@
         <v>17</v>
       </c>
       <c r="U112" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V112" s="4"/>
     </row>
@@ -9293,13 +9293,13 @@
         <v>22</v>
       </c>
       <c r="C113" s="20" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D113" s="14" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F113" s="3">
         <v>6000</v>
@@ -9314,7 +9314,7 @@
         <v>50</v>
       </c>
       <c r="J113" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K113" s="3">
         <v>2</v>
@@ -9349,7 +9349,7 @@
         <v>19</v>
       </c>
       <c r="U113" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V113" s="4"/>
     </row>
@@ -9361,13 +9361,13 @@
         <v>22</v>
       </c>
       <c r="C114" s="20" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D114" s="8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F114" s="3">
         <v>6000</v>
@@ -9382,7 +9382,7 @@
         <v>50</v>
       </c>
       <c r="J114" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K114" s="3">
         <v>2</v>
@@ -9417,7 +9417,7 @@
         <v>19</v>
       </c>
       <c r="U114" s="4" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="V114" s="18"/>
     </row>
@@ -9429,13 +9429,13 @@
         <v>22</v>
       </c>
       <c r="C115" s="20" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D115" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F115" s="3">
         <v>6000</v>
@@ -9450,7 +9450,7 @@
         <v>50</v>
       </c>
       <c r="J115" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K115" s="3">
         <v>2</v>
@@ -9495,13 +9495,13 @@
         <v>22</v>
       </c>
       <c r="C116" s="20" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F116" s="3">
         <v>1000</v>
@@ -9516,7 +9516,7 @@
         <v>70</v>
       </c>
       <c r="J116" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K116" s="3">
         <v>3</v>
@@ -9561,13 +9561,13 @@
         <v>22</v>
       </c>
       <c r="C117" s="20" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D117" s="18" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F117" s="3">
         <v>1000</v>
@@ -9582,7 +9582,7 @@
         <v>70</v>
       </c>
       <c r="J117" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K117" s="3">
         <v>3</v>
@@ -9627,13 +9627,13 @@
         <v>22</v>
       </c>
       <c r="C118" s="20" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D118" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F118" s="3">
         <v>1000</v>
@@ -9648,7 +9648,7 @@
         <v>1000</v>
       </c>
       <c r="J118" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K118" s="3">
         <v>3</v>
@@ -9693,13 +9693,13 @@
         <v>22</v>
       </c>
       <c r="C119" s="20" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F119" s="3">
         <v>1000</v>
@@ -9714,7 +9714,7 @@
         <v>70</v>
       </c>
       <c r="J119" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K119" s="3">
         <v>3</v>
@@ -9759,13 +9759,13 @@
         <v>22</v>
       </c>
       <c r="C120" s="20" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F120" s="3">
         <v>1000</v>
@@ -9780,7 +9780,7 @@
         <v>120</v>
       </c>
       <c r="J120" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K120" s="3">
         <v>3</v>
@@ -9825,13 +9825,13 @@
         <v>22</v>
       </c>
       <c r="C121" s="20" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D121" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F121" s="3">
         <v>1000</v>
@@ -9846,7 +9846,7 @@
         <v>50</v>
       </c>
       <c r="J121" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K121" s="3">
         <v>3</v>
@@ -9891,13 +9891,13 @@
         <v>22</v>
       </c>
       <c r="C122" s="20" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="D122" s="8" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F122" s="3">
         <v>3000</v>
@@ -9957,13 +9957,13 @@
         <v>22</v>
       </c>
       <c r="C123" s="20" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="D123" s="8" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F123" s="3">
         <v>3000</v>
@@ -10023,13 +10023,13 @@
         <v>22</v>
       </c>
       <c r="C124" s="20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D124" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F124" s="3">
         <v>3000</v>
@@ -10089,13 +10089,13 @@
         <v>22</v>
       </c>
       <c r="C125" s="20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D125" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F125" s="3">
         <v>3000</v>
@@ -10155,13 +10155,13 @@
         <v>22</v>
       </c>
       <c r="C126" s="20" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D126" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F126" s="3">
         <v>3000</v>
@@ -10221,13 +10221,13 @@
         <v>22</v>
       </c>
       <c r="C127" s="20" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F127" s="3">
         <v>3000</v>
@@ -10287,13 +10287,13 @@
         <v>22</v>
       </c>
       <c r="C128" s="20" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D128" s="8" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F128" s="3">
         <v>3000</v>
@@ -10353,13 +10353,13 @@
         <v>22</v>
       </c>
       <c r="C129" s="20" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D129" s="8" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F129" s="3">
         <v>3000</v>
@@ -10419,13 +10419,13 @@
         <v>22</v>
       </c>
       <c r="C130" s="20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D130" s="8" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F130" s="3">
         <v>3000</v>
@@ -10467,11 +10467,11 @@
         <v>1</v>
       </c>
       <c r="S130" s="9">
-        <f t="shared" ref="S130:S161" si="9">SUM(K130:R130)</f>
+        <f t="shared" ref="S130:S160" si="9">SUM(K130:R130)</f>
         <v>11</v>
       </c>
       <c r="T130" s="9">
-        <f t="shared" ref="T130:T162" si="10">SUM(K130:Q130)</f>
+        <f t="shared" ref="T130:T161" si="10">SUM(K130:Q130)</f>
         <v>10</v>
       </c>
       <c r="U130" s="21"/>
@@ -10485,13 +10485,13 @@
         <v>22</v>
       </c>
       <c r="C131" s="20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D131" s="8" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F131" s="3">
         <v>3000</v>
@@ -10551,13 +10551,13 @@
         <v>22</v>
       </c>
       <c r="C132" s="20" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D132" s="8" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F132" s="3">
         <v>3000</v>
@@ -10617,13 +10617,13 @@
         <v>22</v>
       </c>
       <c r="C133" s="20" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F133" s="3">
         <v>3000</v>
@@ -10683,13 +10683,13 @@
         <v>22</v>
       </c>
       <c r="C134" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D134" s="8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F134" s="3">
         <v>3000</v>
@@ -10749,13 +10749,13 @@
         <v>22</v>
       </c>
       <c r="C135" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D135" s="8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F135" s="3">
         <v>3000</v>
@@ -10815,13 +10815,13 @@
         <v>22</v>
       </c>
       <c r="C136" s="20" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D136" s="8" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F136" s="3">
         <v>3000</v>
@@ -10881,13 +10881,13 @@
         <v>22</v>
       </c>
       <c r="C137" s="20" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D137" s="8" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="F137" s="3">
         <v>3000</v>
@@ -10902,7 +10902,7 @@
         <v>30</v>
       </c>
       <c r="J137" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K137" s="3">
         <v>3</v>
@@ -10947,13 +10947,13 @@
         <v>22</v>
       </c>
       <c r="C138" s="20" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F138" s="3">
         <v>3000</v>
@@ -10968,7 +10968,7 @@
         <v>210</v>
       </c>
       <c r="J138" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K138" s="3">
         <v>8</v>
@@ -11003,7 +11003,7 @@
         <v>23</v>
       </c>
       <c r="U138" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V138" s="18"/>
     </row>
@@ -11015,13 +11015,13 @@
         <v>22</v>
       </c>
       <c r="C139" s="20" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="D139" s="18" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F139" s="3">
         <v>3000</v>
@@ -11036,7 +11036,7 @@
         <v>210</v>
       </c>
       <c r="J139" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K139" s="3">
         <v>8</v>
@@ -11071,7 +11071,7 @@
         <v>23</v>
       </c>
       <c r="U139" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V139" s="18"/>
     </row>
@@ -11083,13 +11083,13 @@
         <v>22</v>
       </c>
       <c r="C140" s="20" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="D140" s="18" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F140" s="3">
         <v>3000</v>
@@ -11104,7 +11104,7 @@
         <v>210</v>
       </c>
       <c r="J140" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K140" s="3">
         <v>8</v>
@@ -11139,7 +11139,7 @@
         <v>23</v>
       </c>
       <c r="U140" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V140" s="18"/>
     </row>
@@ -11151,13 +11151,13 @@
         <v>22</v>
       </c>
       <c r="C141" s="25" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D141" s="18" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F141" s="3">
         <v>3000</v>
@@ -11172,7 +11172,7 @@
         <v>210</v>
       </c>
       <c r="J141" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K141" s="3">
         <v>8</v>
@@ -11207,7 +11207,7 @@
         <v>23</v>
       </c>
       <c r="U141" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V141" s="4"/>
     </row>
@@ -11219,13 +11219,13 @@
         <v>22</v>
       </c>
       <c r="C142" s="20" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="D142" s="18" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F142" s="3">
         <v>3000</v>
@@ -11240,7 +11240,7 @@
         <v>210</v>
       </c>
       <c r="J142" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K142" s="3">
         <v>8</v>
@@ -11275,7 +11275,7 @@
         <v>23</v>
       </c>
       <c r="U142" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V142" s="4"/>
     </row>
@@ -11287,13 +11287,13 @@
         <v>22</v>
       </c>
       <c r="C143" s="20" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F143" s="3">
         <v>3000</v>
@@ -11308,7 +11308,7 @@
         <v>210</v>
       </c>
       <c r="J143" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K143" s="3">
         <v>8</v>
@@ -11343,7 +11343,7 @@
         <v>23</v>
       </c>
       <c r="U143" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V143" s="18"/>
     </row>
@@ -11355,13 +11355,13 @@
         <v>22</v>
       </c>
       <c r="C144" s="20" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="D144" s="18" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F144" s="3">
         <v>3000</v>
@@ -11376,7 +11376,7 @@
         <v>210</v>
       </c>
       <c r="J144" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K144" s="3">
         <v>8</v>
@@ -11411,7 +11411,7 @@
         <v>23</v>
       </c>
       <c r="U144" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V144" s="18"/>
     </row>
@@ -11423,13 +11423,13 @@
         <v>22</v>
       </c>
       <c r="C145" s="20" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D145" s="18" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="F145" s="3">
         <v>3000</v>
@@ -11444,7 +11444,7 @@
         <v>210</v>
       </c>
       <c r="J145" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K145" s="3">
         <v>8</v>
@@ -11479,7 +11479,7 @@
         <v>23</v>
       </c>
       <c r="U145" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="V145" s="18"/>
     </row>
@@ -12013,25 +12013,25 @@
     </row>
     <row r="154" spans="1:22" ht="13" customHeight="1">
       <c r="A154" s="1">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B154" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C154" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="D154" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E154" s="3" t="s">
-        <v>25</v>
+      <c r="D154" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E154" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="F154" s="3">
         <v>200</v>
       </c>
-      <c r="G154" s="3" t="s">
-        <v>33</v>
+      <c r="G154" s="3">
+        <v>200</v>
       </c>
       <c r="H154" s="3">
         <v>200</v>
@@ -12079,37 +12079,37 @@
     </row>
     <row r="155" spans="1:22" ht="13" customHeight="1">
       <c r="A155" s="1">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B155" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C155" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D155" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E155" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="E155" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="F155" s="3">
         <v>200</v>
       </c>
-      <c r="G155" s="3">
-        <v>200</v>
+      <c r="G155" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="H155" s="3">
         <v>200</v>
       </c>
       <c r="I155" s="8">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="J155" s="8" t="s">
         <v>26</v>
       </c>
       <c r="K155" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L155" s="3">
         <v>1</v>
@@ -12118,46 +12118,46 @@
         <v>0.5</v>
       </c>
       <c r="N155" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O155" s="3">
         <v>0</v>
       </c>
       <c r="P155" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q155" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="R155" s="9">
         <v>0.25</v>
       </c>
       <c r="S155" s="9">
         <f t="shared" si="9"/>
-        <v>3.25</v>
+        <v>5.75</v>
       </c>
       <c r="T155" s="9">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>5.5</v>
       </c>
       <c r="U155" s="21"/>
       <c r="V155" s="10"/>
     </row>
     <row r="156" spans="1:22" ht="13" customHeight="1">
       <c r="A156" s="1">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B156" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C156" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="D156" s="5" t="s">
         <v>48</v>
       </c>
+      <c r="D156" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="E156" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F156" s="3">
         <v>200</v>
@@ -12169,13 +12169,13 @@
         <v>200</v>
       </c>
       <c r="I156" s="8">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="J156" s="8" t="s">
         <v>26</v>
       </c>
       <c r="K156" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L156" s="3">
         <v>1</v>
@@ -12193,103 +12193,105 @@
         <v>0.5</v>
       </c>
       <c r="Q156" s="3">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="R156" s="9">
         <v>0.25</v>
       </c>
       <c r="S156" s="9">
         <f t="shared" si="9"/>
-        <v>5.75</v>
+        <v>4.25</v>
       </c>
       <c r="T156" s="9">
         <f t="shared" si="10"/>
-        <v>5.5</v>
-      </c>
-      <c r="U156" s="21"/>
+        <v>4</v>
+      </c>
+      <c r="U156" s="15"/>
       <c r="V156" s="10"/>
     </row>
     <row r="157" spans="1:22" ht="13" customHeight="1">
       <c r="A157" s="1">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B157" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C157" s="20" t="s">
-        <v>49</v>
+        <v>262</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="E157" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F157" s="3">
-        <v>200</v>
-      </c>
-      <c r="G157" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H157" s="3">
-        <v>200</v>
-      </c>
-      <c r="I157" s="8">
-        <v>50</v>
-      </c>
-      <c r="J157" s="8" t="s">
-        <v>26</v>
+        <v>263</v>
+      </c>
+      <c r="E157" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="F157" s="1">
+        <v>1000</v>
+      </c>
+      <c r="G157" s="1">
+        <v>300</v>
+      </c>
+      <c r="H157" s="1">
+        <v>750</v>
+      </c>
+      <c r="I157" s="10">
+        <v>25</v>
+      </c>
+      <c r="J157" s="10" t="s">
+        <v>117</v>
       </c>
       <c r="K157" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L157" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M157" s="3">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="N157" s="3">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="O157" s="3">
         <v>0</v>
       </c>
       <c r="P157" s="3">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="Q157" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="R157" s="9">
-        <v>0.25</v>
+        <v>5</v>
+      </c>
+      <c r="R157" s="3">
+        <v>4</v>
       </c>
       <c r="S157" s="9">
         <f t="shared" si="9"/>
-        <v>4.25</v>
+        <v>25</v>
       </c>
       <c r="T157" s="9">
         <f t="shared" si="10"/>
-        <v>4</v>
-      </c>
-      <c r="U157" s="15"/>
-      <c r="V157" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="U157" s="3">
+        <v>29</v>
+      </c>
+      <c r="V157" s="18"/>
     </row>
     <row r="158" spans="1:22" ht="13" customHeight="1">
       <c r="A158" s="1">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B158" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C158" s="20" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E158" s="18" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F158" s="1">
         <v>1000</v>
@@ -12304,7 +12306,7 @@
         <v>25</v>
       </c>
       <c r="J158" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K158" s="3">
         <v>5</v>
@@ -12345,19 +12347,19 @@
     </row>
     <row r="159" spans="1:22" ht="13" customHeight="1">
       <c r="A159" s="1">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B159" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C159" s="20" t="s">
-        <v>270</v>
-      </c>
-      <c r="D159" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="E159" s="18" t="s">
-        <v>269</v>
+        <v>46</v>
+      </c>
+      <c r="D159" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="E159" s="17" t="s">
+        <v>264</v>
       </c>
       <c r="F159" s="1">
         <v>1000</v>
@@ -12366,66 +12368,66 @@
         <v>300</v>
       </c>
       <c r="H159" s="1">
-        <v>750</v>
+        <v>1025</v>
       </c>
       <c r="I159" s="10">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="J159" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K159" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L159" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M159" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N159" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O159" s="3">
         <v>0</v>
       </c>
       <c r="P159" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q159" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R159" s="3">
         <v>4</v>
       </c>
       <c r="S159" s="9">
         <f t="shared" si="9"/>
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="T159" s="9">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="U159" s="3">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="V159" s="18"/>
     </row>
     <row r="160" spans="1:22" ht="13" customHeight="1">
       <c r="A160" s="1">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B160" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C160" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D160" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D160" s="14" t="s">
-        <v>48</v>
-      </c>
       <c r="E160" s="17" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="F160" s="1">
         <v>1000</v>
@@ -12437,10 +12439,10 @@
         <v>1025</v>
       </c>
       <c r="I160" s="10">
-        <v>70</v>
+        <v>1000</v>
       </c>
       <c r="J160" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K160" s="3">
         <v>3</v>
@@ -12461,54 +12463,52 @@
         <v>1</v>
       </c>
       <c r="Q160" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R160" s="3">
         <v>4</v>
       </c>
       <c r="S160" s="9">
         <f t="shared" si="9"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T160" s="9">
         <f t="shared" si="10"/>
-        <v>12</v>
-      </c>
-      <c r="U160" s="3">
-        <v>9</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="U160" s="3"/>
       <c r="V160" s="18"/>
     </row>
     <row r="161" spans="1:22" ht="13" customHeight="1">
       <c r="A161" s="1">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B161" s="18" t="s">
         <v>22</v>
       </c>
       <c r="C161" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="D161" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="E161" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="D161" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="E161" s="18" t="s">
         <v>269</v>
       </c>
       <c r="F161" s="1">
         <v>1000</v>
       </c>
       <c r="G161" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="H161" s="1">
-        <v>1025</v>
+        <v>750</v>
       </c>
       <c r="I161" s="10">
-        <v>1000</v>
+        <v>25</v>
       </c>
       <c r="J161" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K161" s="3">
         <v>3</v>
@@ -12535,84 +12535,18 @@
         <v>4</v>
       </c>
       <c r="S161" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="S161" si="11">SUM(K161:R161)</f>
         <v>17</v>
       </c>
       <c r="T161" s="9">
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="U161" s="3"/>
+      <c r="U161" s="1"/>
       <c r="V161" s="18"/>
     </row>
-    <row r="162" spans="1:22" ht="13" customHeight="1">
-      <c r="A162" s="1">
-        <v>161</v>
-      </c>
-      <c r="B162" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C162" s="20" t="s">
-        <v>272</v>
-      </c>
-      <c r="D162" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="E162" s="18" t="s">
-        <v>274</v>
-      </c>
-      <c r="F162" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G162" s="1">
-        <v>500</v>
-      </c>
-      <c r="H162" s="1">
-        <v>750</v>
-      </c>
-      <c r="I162" s="10">
-        <v>25</v>
-      </c>
-      <c r="J162" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="K162" s="3">
-        <v>3</v>
-      </c>
-      <c r="L162" s="3">
-        <v>2</v>
-      </c>
-      <c r="M162" s="3">
-        <v>1</v>
-      </c>
-      <c r="N162" s="3">
-        <v>1</v>
-      </c>
-      <c r="O162" s="3">
-        <v>0</v>
-      </c>
-      <c r="P162" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q162" s="3">
-        <v>5</v>
-      </c>
-      <c r="R162" s="3">
-        <v>4</v>
-      </c>
-      <c r="S162" s="9">
-        <f t="shared" ref="S162:S193" si="11">SUM(K162:R162)</f>
-        <v>17</v>
-      </c>
-      <c r="T162" s="9">
-        <f t="shared" si="10"/>
-        <v>13</v>
-      </c>
-      <c r="U162" s="1"/>
-      <c r="V162" s="18"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V162"/>
+  <autoFilter ref="A1:V161"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -12631,16 +12565,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="26" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -12648,13 +12582,13 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -12662,13 +12596,13 @@
         <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -12676,13 +12610,13 @@
         <v>141</v>
       </c>
       <c r="B4" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C4" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D4" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>